<commit_message>
Fix year-end close picking the day before 31 December
GetClosingPriceOnDate returned the previous trading day's close whenever
the target date (e.g. 31 December) was itself a trading day. Yahoo's daily
bar timestamp is the intraday market open (~14:30 UTC), stored via
time.Unix as a local-time instant; comparing that afternoon instant against
the target's UTC midnight made the target day look "after" the target and
excluded it.

Fix at ingestion: normalize each bar's timestamp to its UTC calendar date
(valid for US exchanges, whose 09:30 ET open shares the trading date's UTC
day) so PriceData.Date is a real date. This makes GetClosingPriceOnDate
correct and also removes latent timezone fragility in the peak-date and
date-formatting paths.

For real data this shifts the Schedule FA year-end close to 31 December's
value (from 30 December's); golden workbook regenerated.
</commit_message>
<xml_diff>
--- a/test/e2e/testdata/expected.xlsx
+++ b/test/e2e/testdata/expected.xlsx
@@ -785,10 +785,10 @@
         <v>82.72</v>
       </c>
       <c r="U2" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V2" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W2" s="5">
         <v>46022</v>
@@ -806,7 +806,7 @@
         <v>847317.4873388672</v>
       </c>
       <c r="AC2" s="4">
-        <v>450671.12459793093</v>
+        <v>443230.78678344726</v>
       </c>
       <c r="AD2" s="4">
         <v>0</v>
@@ -869,10 +869,10 @@
         <v>82.72</v>
       </c>
       <c r="U3" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V3" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W3" s="5">
         <v>46022</v>
@@ -890,7 +890,7 @@
         <v>1264557.1591345214</v>
       </c>
       <c r="AC3" s="4">
-        <v>672592.5117105484</v>
+        <v>661488.3711843872</v>
       </c>
       <c r="AD3" s="4">
         <v>0</v>
@@ -953,10 +953,10 @@
         <v>82.72</v>
       </c>
       <c r="U4" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V4" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W4" s="5">
         <v>46022</v>
@@ -974,7 +974,7 @@
         <v>770288.6248535156</v>
       </c>
       <c r="AC4" s="4">
-        <v>409701.0223617554</v>
+        <v>402937.078894043</v>
       </c>
       <c r="AD4" s="4">
         <v>0</v>
@@ -1037,10 +1037,10 @@
         <v>82.72</v>
       </c>
       <c r="U5" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V5" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W5" s="5">
         <v>46022</v>
@@ -1058,7 +1058,7 @@
         <v>25676.287495117187</v>
       </c>
       <c r="AC5" s="4">
-        <v>13656.700745391845</v>
+        <v>13431.235963134766</v>
       </c>
       <c r="AD5" s="4">
         <v>0</v>
@@ -1121,10 +1121,10 @@
         <v>82.72</v>
       </c>
       <c r="U6" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V6" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W6" s="5">
         <v>46022</v>
@@ -1142,7 +1142,7 @@
         <v>1168271.081027832</v>
       </c>
       <c r="AC6" s="4">
-        <v>621379.883915329</v>
+        <v>611121.2363226318</v>
       </c>
       <c r="AD6" s="4">
         <v>0</v>
@@ -1205,10 +1205,10 @@
         <v>82.72</v>
       </c>
       <c r="U7" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V7" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W7" s="5">
         <v>46022</v>
@@ -1226,7 +1226,7 @@
         <v>699678.8342419433</v>
       </c>
       <c r="AC7" s="4">
-        <v>372145.0953119278</v>
+        <v>366001.17999542237</v>
       </c>
       <c r="AD7" s="4">
         <v>0</v>
@@ -1289,10 +1289,10 @@
         <v>82.72</v>
       </c>
       <c r="U8" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V8" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W8" s="5">
         <v>46022</v>
@@ -1310,7 +1310,7 @@
         <v>1270976.2310083008</v>
       </c>
       <c r="AC8" s="4">
-        <v>676006.6868968963</v>
+        <v>664846.1801751709</v>
       </c>
       <c r="AD8" s="4">
         <v>0</v>
@@ -1373,10 +1373,10 @@
         <v>82.72</v>
       </c>
       <c r="U9" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V9" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W9" s="5">
         <v>46022</v>
@@ -1394,7 +1394,7 @@
         <v>770288.6248535156</v>
       </c>
       <c r="AC9" s="4">
-        <v>409701.0223617554</v>
+        <v>402937.078894043</v>
       </c>
       <c r="AD9" s="4">
         <v>0</v>
@@ -1457,10 +1457,10 @@
         <v>82.72</v>
       </c>
       <c r="U10" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V10" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W10" s="5">
         <v>46022</v>
@@ -1478,7 +1478,7 @@
         <v>783126.7686010742</v>
       </c>
       <c r="AC10" s="4">
-        <v>416529.3727344513</v>
+        <v>409652.69687561033</v>
       </c>
       <c r="AD10" s="4">
         <v>0</v>
@@ -1541,10 +1541,10 @@
         <v>82.72</v>
       </c>
       <c r="U11" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V11" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W11" s="5">
         <v>46022</v>
@@ -1562,7 +1562,7 @@
         <v>211829.3718347168</v>
       </c>
       <c r="AC11" s="4">
-        <v>112667.78114948273</v>
+        <v>110807.69669586181</v>
       </c>
       <c r="AD11" s="4">
         <v>0</v>
@@ -1625,10 +1625,10 @@
         <v>82.72</v>
       </c>
       <c r="U12" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V12" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W12" s="5">
         <v>46022</v>
@@ -1646,7 +1646,7 @@
         <v>391563.3843005371</v>
       </c>
       <c r="AC12" s="4">
-        <v>208264.68636722566</v>
+        <v>204826.34843780517</v>
       </c>
       <c r="AD12" s="4">
         <v>0</v>
@@ -1709,10 +1709,10 @@
         <v>82.72</v>
       </c>
       <c r="U13" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V13" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W13" s="5">
         <v>46022</v>
@@ -1730,7 +1730,7 @@
         <v>1052727.7872998046</v>
       </c>
       <c r="AC13" s="4">
-        <v>559924.7305610657</v>
+        <v>550680.6744885254</v>
       </c>
       <c r="AD13" s="4">
         <v>0</v>
@@ -1793,10 +1793,10 @@
         <v>82.72</v>
       </c>
       <c r="U14" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V14" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W14" s="5">
         <v>46022</v>
@@ -1814,7 +1814,7 @@
         <v>224667.51558227537</v>
       </c>
       <c r="AC14" s="4">
-        <v>119496.13152217865</v>
+        <v>117523.3146774292</v>
       </c>
       <c r="AD14" s="4">
         <v>0</v>
@@ -1877,10 +1877,10 @@
         <v>86.2</v>
       </c>
       <c r="U15" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V15" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W15" s="5">
         <v>46022</v>
@@ -1898,7 +1898,7 @@
         <v>523251.6862838745</v>
       </c>
       <c r="AC15" s="4">
-        <v>283376.5404668808</v>
+        <v>278698.1462350464</v>
       </c>
       <c r="AD15" s="4">
         <v>0</v>
@@ -1961,10 +1961,10 @@
         <v>86.2</v>
       </c>
       <c r="U16" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V16" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W16" s="5">
         <v>46022</v>
@@ -1982,7 +1982,7 @@
         <v>882593.2057800293</v>
       </c>
       <c r="AC16" s="4">
-        <v>477984.5260887146</v>
+        <v>470093.2587097168</v>
       </c>
       <c r="AD16" s="4">
         <v>0</v>
@@ -2045,10 +2045,10 @@
         <v>86.2</v>
       </c>
       <c r="U17" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V17" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W17" s="5">
         <v>46022</v>
@@ -2066,7 +2066,7 @@
         <v>384558.4682327271</v>
       </c>
       <c r="AC17" s="4">
-        <v>208264.68636722566</v>
+        <v>204826.34843780517</v>
       </c>
       <c r="AD17" s="4">
         <v>0</v>
@@ -2129,10 +2129,10 @@
         <v>86.2</v>
       </c>
       <c r="U18" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V18" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W18" s="5">
         <v>46022</v>
@@ -2150,7 +2150,7 @@
         <v>315211.8592071533</v>
       </c>
       <c r="AC18" s="4">
-        <v>170708.75931739807</v>
+        <v>167890.44953918457</v>
       </c>
       <c r="AD18" s="4">
         <v>0</v>
@@ -2213,10 +2213,10 @@
         <v>86.2</v>
       </c>
       <c r="U19" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V19" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W19" s="5">
         <v>46022</v>
@@ -2234,7 +2234,7 @@
         <v>479122.0259948731</v>
       </c>
       <c r="AC19" s="4">
-        <v>259477.31416244505</v>
+        <v>255193.48329956055</v>
       </c>
       <c r="AD19" s="4">
         <v>0</v>
@@ -2297,10 +2297,10 @@
         <v>86.2</v>
       </c>
       <c r="U20" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V20" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W20" s="5">
         <v>46022</v>
@@ -2318,7 +2318,7 @@
         <v>1204109.3021713258</v>
       </c>
       <c r="AC20" s="4">
-        <v>652107.4605924606</v>
+        <v>641341.517239685</v>
       </c>
       <c r="AD20" s="4">
         <v>0</v>
@@ -2381,10 +2381,10 @@
         <v>86.2</v>
       </c>
       <c r="U21" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V21" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W21" s="5">
         <v>46022</v>
@@ -2402,7 +2402,7 @@
         <v>882593.2057800293</v>
       </c>
       <c r="AC21" s="4">
-        <v>477984.5260887146</v>
+        <v>470093.2587097168</v>
       </c>
       <c r="AD21" s="4">
         <v>0</v>
@@ -2465,10 +2465,10 @@
         <v>86.2</v>
       </c>
       <c r="U22" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V22" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W22" s="5">
         <v>46022</v>
@@ -2486,7 +2486,7 @@
         <v>308907.6220230103</v>
       </c>
       <c r="AC22" s="4">
-        <v>167294.5841310501</v>
+        <v>164532.64054840087</v>
       </c>
       <c r="AD22" s="4">
         <v>0</v>
@@ -2549,10 +2549,10 @@
         <v>86.2</v>
       </c>
       <c r="U23" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V23" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W23" s="5">
         <v>46022</v>
@@ -2570,7 +2570,7 @@
         <v>138693.21805114747</v>
       </c>
       <c r="AC23" s="4">
-        <v>75111.85409965515</v>
+        <v>73871.7977972412</v>
       </c>
       <c r="AD23" s="4">
         <v>0</v>
@@ -2633,10 +2633,10 @@
         <v>86.2</v>
       </c>
       <c r="U24" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V24" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W24" s="5">
         <v>46022</v>
@@ -2654,7 +2654,7 @@
         <v>37825.4231048584</v>
       </c>
       <c r="AC24" s="4">
-        <v>20485.05111808777</v>
+        <v>20146.853944702147</v>
       </c>
       <c r="AD24" s="4">
         <v>0</v>
@@ -2717,10 +2717,10 @@
         <v>86.2</v>
       </c>
       <c r="U25" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V25" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W25" s="5">
         <v>46022</v>
@@ -2738,7 +2738,7 @@
         <v>598902.5324935913</v>
       </c>
       <c r="AC25" s="4">
-        <v>324346.64270305634</v>
+        <v>318991.8541244507</v>
       </c>
       <c r="AD25" s="4">
         <v>0</v>
@@ -2801,10 +2801,10 @@
         <v>86.2</v>
       </c>
       <c r="U26" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V26" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W26" s="5">
         <v>46022</v>
@@ -2822,7 +2822,7 @@
         <v>863680.4942276002</v>
       </c>
       <c r="AC26" s="4">
-        <v>467742.0005296707</v>
+        <v>460019.8317373657</v>
       </c>
       <c r="AD26" s="4">
         <v>0</v>
@@ -2885,10 +2885,10 @@
         <v>86.2</v>
       </c>
       <c r="U27" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V27" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W27" s="5">
         <v>46022</v>
@@ -2906,7 +2906,7 @@
         <v>1185196.5906188965</v>
       </c>
       <c r="AC27" s="4">
-        <v>641864.9350334167</v>
+        <v>631268.090267334</v>
       </c>
       <c r="AD27" s="4">
         <v>0</v>
@@ -2969,10 +2969,10 @@
         <v>86.2</v>
       </c>
       <c r="U28" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V28" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W28" s="5">
         <v>46022</v>
@@ -2990,7 +2990,7 @@
         <v>781725.4108337403</v>
       </c>
       <c r="AC28" s="4">
-        <v>423357.7231071472</v>
+        <v>416368.3148571777</v>
       </c>
       <c r="AD28" s="4">
         <v>0</v>
@@ -3053,10 +3053,10 @@
         <v>84.25</v>
       </c>
       <c r="U29" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V29" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W29" s="5">
         <v>46022</v>
@@ -3074,7 +3074,7 @@
         <v>432141.8424682617</v>
       </c>
       <c r="AC29" s="4">
-        <v>327760.8178894043</v>
+        <v>322349.66311523435</v>
       </c>
       <c r="AD29" s="4">
         <v>0</v>
@@ -3137,10 +3137,10 @@
         <v>84.25</v>
       </c>
       <c r="U30" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V30" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W30" s="5">
         <v>46022</v>
@@ -3158,7 +3158,7 @@
         <v>846277.7748336792</v>
       </c>
       <c r="AC30" s="4">
-        <v>641864.9350334167</v>
+        <v>631268.090267334</v>
       </c>
       <c r="AD30" s="4">
         <v>0</v>
@@ -3221,10 +3221,10 @@
         <v>84.25</v>
       </c>
       <c r="U31" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V31" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W31" s="5">
         <v>46022</v>
@@ -3242,7 +3242,7 @@
         <v>720236.4041137695</v>
       </c>
       <c r="AC31" s="4">
-        <v>546268.0298156738</v>
+        <v>537249.4385253906</v>
       </c>
       <c r="AD31" s="4">
         <v>0</v>
@@ -3305,10 +3305,10 @@
         <v>88.2</v>
       </c>
       <c r="U32" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V32" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W32" s="5">
         <v>46022</v>
@@ -3326,7 +3326,7 @@
         <v>130550.11434173584</v>
       </c>
       <c r="AC32" s="4">
-        <v>99011.08040409088</v>
+        <v>97376.46073272705</v>
       </c>
       <c r="AD32" s="4">
         <v>0</v>
@@ -3389,10 +3389,10 @@
         <v>88.2</v>
       </c>
       <c r="U33" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V33" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W33" s="5">
         <v>46022</v>
@@ -3410,7 +3410,7 @@
         <v>72027.64929199219</v>
       </c>
       <c r="AC33" s="4">
-        <v>54626.80298156738</v>
+        <v>53724.943852539065</v>
       </c>
       <c r="AD33" s="4">
         <v>0</v>
@@ -3473,10 +3473,10 @@
         <v>88.2</v>
       </c>
       <c r="U34" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V34" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W34" s="5">
         <v>46022</v>
@@ -3494,7 +3494,7 @@
         <v>486186.63272094727</v>
       </c>
       <c r="AC34" s="4">
-        <v>368730.9201255798</v>
+        <v>362643.37100463867</v>
       </c>
       <c r="AD34" s="4">
         <v>0</v>
@@ -3557,10 +3557,10 @@
         <v>88.2</v>
       </c>
       <c r="U35" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V35" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W35" s="5">
         <v>46022</v>
@@ -3578,7 +3578,7 @@
         <v>76529.3773727417</v>
       </c>
       <c r="AC35" s="4">
-        <v>58040.978167915346</v>
+        <v>57082.752843322756</v>
       </c>
       <c r="AD35" s="4">
         <v>0</v>
@@ -3641,10 +3641,10 @@
         <v>88.2</v>
       </c>
       <c r="U36" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V36" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W36" s="5">
         <v>46022</v>
@@ -3662,7 +3662,7 @@
         <v>612235.0189819336</v>
       </c>
       <c r="AC36" s="4">
-        <v>464327.82534332277</v>
+        <v>456662.02274658205</v>
       </c>
       <c r="AD36" s="4">
         <v>0</v>
@@ -3725,10 +3725,10 @@
         <v>88.2</v>
       </c>
       <c r="U37" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V37" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W37" s="5">
         <v>46022</v>
@@ -3746,7 +3746,7 @@
         <v>801307.5983734131</v>
       </c>
       <c r="AC37" s="4">
-        <v>607723.1831699371</v>
+        <v>597690.000359497</v>
       </c>
       <c r="AD37" s="4">
         <v>0</v>
@@ -3809,10 +3809,10 @@
         <v>88.2</v>
       </c>
       <c r="U38" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V38" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W38" s="5">
         <v>46022</v>
@@ -3830,7 +3830,7 @@
         <v>571719.466255188</v>
       </c>
       <c r="AC38" s="4">
-        <v>433600.2486661911</v>
+        <v>426441.7418295288</v>
       </c>
       <c r="AD38" s="4">
         <v>0</v>
@@ -3893,10 +3893,10 @@
         <v>88.2</v>
       </c>
       <c r="U39" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V39" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W39" s="5">
         <v>46022</v>
@@ -3914,7 +3914,7 @@
         <v>450172.8080749512</v>
       </c>
       <c r="AC39" s="4">
-        <v>341417.51863479614</v>
+        <v>335780.89907836914</v>
       </c>
       <c r="AD39" s="4">
         <v>0</v>
@@ -3977,10 +3977,10 @@
         <v>88.2</v>
       </c>
       <c r="U40" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V40" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W40" s="5">
         <v>46022</v>
@@ -3998,7 +3998,7 @@
         <v>216082.94787597656</v>
       </c>
       <c r="AC40" s="4">
-        <v>163880.40894470215</v>
+        <v>161174.83155761717</v>
       </c>
       <c r="AD40" s="4">
         <v>0</v>
@@ -4061,10 +4061,10 @@
         <v>88.95</v>
       </c>
       <c r="U41" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V41" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W41" s="5">
         <v>46022</v>
@@ -4082,7 +4082,7 @@
         <v>293241.4704969406</v>
       </c>
       <c r="AC41" s="4">
-        <v>276548.1900941849</v>
+        <v>271982.528253479</v>
       </c>
       <c r="AD41" s="4">
         <v>0</v>
@@ -4145,10 +4145,10 @@
         <v>88.95</v>
       </c>
       <c r="U42" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V42" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W42" s="5">
         <v>46022</v>
@@ -4166,7 +4166,7 @@
         <v>130438.05951576233</v>
       </c>
       <c r="AC42" s="4">
-        <v>129738.65708122253</v>
+        <v>127596.74164978028</v>
       </c>
       <c r="AD42" s="4">
         <v>0</v>
@@ -4229,10 +4229,10 @@
         <v>88.95</v>
       </c>
       <c r="U43" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V43" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W43" s="5">
         <v>46022</v>
@@ -4250,7 +4250,7 @@
         <v>133870.64002933502</v>
       </c>
       <c r="AC43" s="4">
-        <v>133152.83226757048</v>
+        <v>130954.55064056396</v>
       </c>
       <c r="AD43" s="4">
         <v>0</v>
@@ -4313,10 +4313,10 @@
         <v>88.95</v>
       </c>
       <c r="U44" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V44" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W44" s="5">
         <v>46022</v>
@@ -4334,7 +4334,7 @@
         <v>494291.5939544678</v>
       </c>
       <c r="AC44" s="4">
-        <v>491641.22683410643</v>
+        <v>483524.4946728516</v>
       </c>
       <c r="AD44" s="4">
         <v>0</v>
@@ -4397,10 +4397,10 @@
         <v>88.95</v>
       </c>
       <c r="U45" s="5">
-        <v>46021</v>
+        <v>46022</v>
       </c>
       <c r="V45" s="3">
-        <v>38.15999984741211</v>
+        <v>37.529998779296875</v>
       </c>
       <c r="W45" s="5">
         <v>46022</v>
@@ -4418,7 +4418,7 @@
         <v>219685.15286865234</v>
       </c>
       <c r="AC45" s="4">
-        <v>218507.21192626952</v>
+        <v>214899.77541015626</v>
       </c>
       <c r="AD45" s="4">
         <v>0</v>

</xml_diff>